<commit_message>
Fase 4: cierre de resultados del dia
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -542,6 +542,25 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>